<commit_message>
ajustes e criação do ajustar serial instrumento depois das duplicações
</commit_message>
<xml_diff>
--- a/cadastrar.xlsx
+++ b/cadastrar.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\gitlocal\protheus\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3A14F2EA-E760-4B3C-A136-708E9736D8A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B7BCE3F-7BFF-4C0D-BC0D-44ED8B3CED23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1590" yWindow="150" windowWidth="18900" windowHeight="10800" xr2:uid="{1589334F-D7EF-4C27-A54A-7D2B83ACDBA2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{1589334F-D7EF-4C27-A54A-7D2B83ACDBA2}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1174" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1179" uniqueCount="150">
   <si>
     <t>CLIENTE</t>
   </si>
@@ -474,6 +474,21 @@
   </si>
   <si>
     <t>8000ZE</t>
+  </si>
+  <si>
+    <t>COD_CONTATO</t>
+  </si>
+  <si>
+    <t>CLASSIFIC</t>
+  </si>
+  <si>
+    <t>OCORRENCIA</t>
+  </si>
+  <si>
+    <t>MEMO</t>
+  </si>
+  <si>
+    <t>ACESSORIOS</t>
   </si>
 </sst>
 </file>
@@ -522,7 +537,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -550,6 +565,21 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -885,11 +915,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7600A1C-8D91-4C3A-A5DE-920816BE31C1}">
-  <dimension ref="A1:T100"/>
+  <dimension ref="A1:Y100"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.28515625" style="18" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="17.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="21.5703125" bestFit="1" customWidth="1"/>
@@ -907,13 +937,15 @@
     <col min="18" max="18" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="6.28515625" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="19.140625" customWidth="1"/>
+    <col min="22" max="22" width="17.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="14" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -970,12 +1002,27 @@
       <c r="T1" s="3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U1" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C2" s="11" t="s">
@@ -1032,11 +1079,11 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C3" s="11" t="s">
@@ -1093,11 +1140,11 @@
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C4" s="11" t="s">
@@ -1154,11 +1201,11 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C5" s="11" t="s">
@@ -1215,11 +1262,11 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C6" s="11" t="s">
@@ -1276,11 +1323,11 @@
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C7" s="11" t="s">
@@ -1337,11 +1384,11 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C8" s="11" t="s">
@@ -1398,11 +1445,11 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C9" s="11" t="s">
@@ -1459,11 +1506,11 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C10" s="11" t="s">
@@ -1520,11 +1567,11 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C11" s="11" t="s">
@@ -1581,11 +1628,11 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C12" s="11" t="s">
@@ -1642,11 +1689,11 @@
         <v>39</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C13" s="11" t="s">
@@ -1703,11 +1750,11 @@
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C14" s="11" t="s">
@@ -1764,11 +1811,11 @@
         <v>41</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C15" s="11" t="s">
@@ -1825,11 +1872,11 @@
         <v>42</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C16" s="11" t="s">
@@ -1890,7 +1937,7 @@
       <c r="A17" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C17" s="11" t="s">
@@ -1951,7 +1998,7 @@
       <c r="A18" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="B18" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C18" s="11" t="s">
@@ -2012,7 +2059,7 @@
       <c r="A19" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="B19" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C19" s="11" t="s">
@@ -2073,7 +2120,7 @@
       <c r="A20" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="B20" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C20" s="11" t="s">
@@ -2134,7 +2181,7 @@
       <c r="A21" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B21" s="8" t="s">
+      <c r="B21" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C21" s="11" t="s">
@@ -2195,7 +2242,7 @@
       <c r="A22" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="B22" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C22" s="11" t="s">
@@ -2256,7 +2303,7 @@
       <c r="A23" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B23" s="8" t="s">
+      <c r="B23" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C23" s="11" t="s">
@@ -2317,7 +2364,7 @@
       <c r="A24" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C24" s="11" t="s">
@@ -2378,7 +2425,7 @@
       <c r="A25" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C25" s="11" t="s">
@@ -2439,7 +2486,7 @@
       <c r="A26" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C26" s="11" t="s">
@@ -2500,7 +2547,7 @@
       <c r="A27" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B27" s="8" t="s">
+      <c r="B27" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C27" s="11" t="s">
@@ -2561,7 +2608,7 @@
       <c r="A28" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B28" s="8" t="s">
+      <c r="B28" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C28" s="11" t="s">
@@ -2622,7 +2669,7 @@
       <c r="A29" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B29" s="8" t="s">
+      <c r="B29" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C29" s="11" t="s">
@@ -2683,7 +2730,7 @@
       <c r="A30" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B30" s="8" t="s">
+      <c r="B30" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C30" s="11" t="s">
@@ -2744,7 +2791,7 @@
       <c r="A31" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B31" s="8" t="s">
+      <c r="B31" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C31" s="11" t="s">
@@ -2805,7 +2852,7 @@
       <c r="A32" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B32" s="8" t="s">
+      <c r="B32" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C32" s="11" t="s">
@@ -2866,7 +2913,7 @@
       <c r="A33" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B33" s="8" t="s">
+      <c r="B33" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C33" s="11" t="s">
@@ -2927,7 +2974,7 @@
       <c r="A34" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B34" s="8" t="s">
+      <c r="B34" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C34" s="11" t="s">
@@ -2988,7 +3035,7 @@
       <c r="A35" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B35" s="8" t="s">
+      <c r="B35" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C35" s="11" t="s">
@@ -3049,7 +3096,7 @@
       <c r="A36" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B36" s="8" t="s">
+      <c r="B36" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C36" s="11" t="s">
@@ -3110,7 +3157,7 @@
       <c r="A37" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B37" s="8" t="s">
+      <c r="B37" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C37" s="11" t="s">
@@ -3171,7 +3218,7 @@
       <c r="A38" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B38" s="8" t="s">
+      <c r="B38" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C38" s="11" t="s">
@@ -3232,7 +3279,7 @@
       <c r="A39" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B39" s="8" t="s">
+      <c r="B39" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C39" s="11" t="s">
@@ -3293,7 +3340,7 @@
       <c r="A40" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B40" s="8" t="s">
+      <c r="B40" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C40" s="11" t="s">
@@ -3354,7 +3401,7 @@
       <c r="A41" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B41" s="8" t="s">
+      <c r="B41" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C41" s="11" t="s">
@@ -3415,7 +3462,7 @@
       <c r="A42" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B42" s="8" t="s">
+      <c r="B42" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C42" s="11" t="s">
@@ -3476,7 +3523,7 @@
       <c r="A43" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B43" s="8" t="s">
+      <c r="B43" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C43" s="11" t="s">
@@ -3537,7 +3584,7 @@
       <c r="A44" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B44" s="8" t="s">
+      <c r="B44" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C44" s="11" t="s">
@@ -3598,7 +3645,7 @@
       <c r="A45" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B45" s="8" t="s">
+      <c r="B45" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C45" s="11" t="s">
@@ -3659,7 +3706,7 @@
       <c r="A46" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B46" s="8" t="s">
+      <c r="B46" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C46" s="11" t="s">
@@ -3720,7 +3767,7 @@
       <c r="A47" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B47" s="8" t="s">
+      <c r="B47" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C47" s="11" t="s">
@@ -3781,7 +3828,7 @@
       <c r="A48" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B48" s="8" t="s">
+      <c r="B48" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C48" s="11" t="s">
@@ -3842,7 +3889,7 @@
       <c r="A49" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B49" s="8" t="s">
+      <c r="B49" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C49" s="11" t="s">
@@ -3903,7 +3950,7 @@
       <c r="A50" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B50" s="8" t="s">
+      <c r="B50" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C50" s="11" t="s">
@@ -3964,7 +4011,7 @@
       <c r="A51" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B51" s="8" t="s">
+      <c r="B51" s="15" t="s">
         <v>136</v>
       </c>
       <c r="C51" s="11" t="s">
@@ -4025,7 +4072,7 @@
       <c r="A52" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="B52" s="8">
+      <c r="B52" s="15">
         <v>11</v>
       </c>
       <c r="C52" s="11" t="s">
@@ -4086,7 +4133,7 @@
       <c r="A53" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="B53" s="8">
+      <c r="B53" s="15">
         <v>11</v>
       </c>
       <c r="C53" s="11" t="s">
@@ -4147,7 +4194,7 @@
       <c r="A54" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="B54" s="8">
+      <c r="B54" s="15">
         <v>11</v>
       </c>
       <c r="C54" s="11" t="s">
@@ -4208,7 +4255,7 @@
       <c r="A55" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="B55" s="8">
+      <c r="B55" s="15">
         <v>11</v>
       </c>
       <c r="C55" s="11" t="s">
@@ -4269,7 +4316,7 @@
       <c r="A56" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="B56" s="8">
+      <c r="B56" s="15">
         <v>11</v>
       </c>
       <c r="C56" s="11" t="s">
@@ -4330,7 +4377,7 @@
       <c r="A57" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="B57" s="8">
+      <c r="B57" s="15">
         <v>11</v>
       </c>
       <c r="C57" s="11" t="s">
@@ -4391,7 +4438,7 @@
       <c r="A58" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="B58" s="8">
+      <c r="B58" s="15">
         <v>11</v>
       </c>
       <c r="C58" s="11" t="s">
@@ -4452,7 +4499,7 @@
       <c r="A59" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="B59" s="8">
+      <c r="B59" s="15">
         <v>11</v>
       </c>
       <c r="C59" s="11" t="s">
@@ -4513,7 +4560,7 @@
       <c r="A60" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="B60" s="8">
+      <c r="B60" s="15">
         <v>11</v>
       </c>
       <c r="C60" s="11" t="s">
@@ -4574,7 +4621,7 @@
       <c r="A61" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="B61" s="8">
+      <c r="B61" s="15">
         <v>11</v>
       </c>
       <c r="C61" s="11" t="s">
@@ -4635,7 +4682,7 @@
       <c r="A62" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="B62" s="8" t="s">
+      <c r="B62" s="15" t="s">
         <v>139</v>
       </c>
       <c r="C62" s="11" t="s">
@@ -4696,7 +4743,7 @@
       <c r="A63" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="B63" s="8" t="s">
+      <c r="B63" s="15" t="s">
         <v>139</v>
       </c>
       <c r="C63" s="11" t="s">
@@ -4757,7 +4804,7 @@
       <c r="A64" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="B64" s="8" t="s">
+      <c r="B64" s="15" t="s">
         <v>139</v>
       </c>
       <c r="C64" s="11" t="s">
@@ -4818,7 +4865,7 @@
       <c r="A65" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="B65" s="8" t="s">
+      <c r="B65" s="15" t="s">
         <v>139</v>
       </c>
       <c r="C65" s="11" t="s">
@@ -4879,7 +4926,7 @@
       <c r="A66" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="B66" s="8" t="s">
+      <c r="B66" s="15" t="s">
         <v>139</v>
       </c>
       <c r="C66" s="11" t="s">
@@ -4940,7 +4987,7 @@
       <c r="A67" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="B67" s="8" t="s">
+      <c r="B67" s="15" t="s">
         <v>139</v>
       </c>
       <c r="C67" s="11" t="s">
@@ -5001,7 +5048,7 @@
       <c r="A68" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="B68" s="8" t="s">
+      <c r="B68" s="15" t="s">
         <v>139</v>
       </c>
       <c r="C68" s="11" t="s">
@@ -5062,7 +5109,7 @@
       <c r="A69" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="B69" s="8" t="s">
+      <c r="B69" s="15" t="s">
         <v>139</v>
       </c>
       <c r="C69" s="11" t="s">
@@ -5123,7 +5170,7 @@
       <c r="A70" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="B70" s="8" t="s">
+      <c r="B70" s="15" t="s">
         <v>139</v>
       </c>
       <c r="C70" s="11" t="s">
@@ -5184,7 +5231,7 @@
       <c r="A71" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="B71" s="8" t="s">
+      <c r="B71" s="15" t="s">
         <v>139</v>
       </c>
       <c r="C71" s="11" t="s">
@@ -5245,7 +5292,7 @@
       <c r="A72" s="11" t="s">
         <v>141</v>
       </c>
-      <c r="B72" s="11" t="s">
+      <c r="B72" s="16" t="s">
         <v>138</v>
       </c>
       <c r="C72" s="11" t="s">
@@ -5306,7 +5353,7 @@
       <c r="A73" s="11" t="s">
         <v>141</v>
       </c>
-      <c r="B73" s="11" t="s">
+      <c r="B73" s="16" t="s">
         <v>138</v>
       </c>
       <c r="C73" s="11" t="s">
@@ -5367,7 +5414,7 @@
       <c r="A74" s="11" t="s">
         <v>141</v>
       </c>
-      <c r="B74" s="11" t="s">
+      <c r="B74" s="16" t="s">
         <v>138</v>
       </c>
       <c r="C74" s="11" t="s">
@@ -5428,7 +5475,7 @@
       <c r="A75" s="11" t="s">
         <v>141</v>
       </c>
-      <c r="B75" s="11" t="s">
+      <c r="B75" s="16" t="s">
         <v>138</v>
       </c>
       <c r="C75" s="11" t="s">
@@ -5489,7 +5536,7 @@
       <c r="A76" s="11" t="s">
         <v>141</v>
       </c>
-      <c r="B76" s="11" t="s">
+      <c r="B76" s="16" t="s">
         <v>138</v>
       </c>
       <c r="C76" s="11" t="s">
@@ -5550,7 +5597,7 @@
       <c r="A77" s="11" t="s">
         <v>141</v>
       </c>
-      <c r="B77" s="11" t="s">
+      <c r="B77" s="16" t="s">
         <v>138</v>
       </c>
       <c r="C77" s="11" t="s">
@@ -5611,7 +5658,7 @@
       <c r="A78" s="11" t="s">
         <v>141</v>
       </c>
-      <c r="B78" s="11" t="s">
+      <c r="B78" s="16" t="s">
         <v>138</v>
       </c>
       <c r="C78" s="11" t="s">
@@ -5672,7 +5719,7 @@
       <c r="A79" s="11" t="s">
         <v>141</v>
       </c>
-      <c r="B79" s="11" t="s">
+      <c r="B79" s="16" t="s">
         <v>138</v>
       </c>
       <c r="C79" s="11" t="s">
@@ -5733,7 +5780,7 @@
       <c r="A80" s="11" t="s">
         <v>141</v>
       </c>
-      <c r="B80" s="11" t="s">
+      <c r="B80" s="16" t="s">
         <v>138</v>
       </c>
       <c r="C80" s="11" t="s">
@@ -5794,7 +5841,7 @@
       <c r="A81" s="11" t="s">
         <v>141</v>
       </c>
-      <c r="B81" s="11" t="s">
+      <c r="B81" s="16" t="s">
         <v>138</v>
       </c>
       <c r="C81" s="11" t="s">
@@ -5855,7 +5902,7 @@
       <c r="A82" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="B82" s="10" t="s">
+      <c r="B82" s="17" t="s">
         <v>136</v>
       </c>
       <c r="C82" s="11" t="s">
@@ -5916,7 +5963,7 @@
       <c r="A83" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="B83" s="10" t="s">
+      <c r="B83" s="17" t="s">
         <v>136</v>
       </c>
       <c r="C83" s="11" t="s">
@@ -5977,7 +6024,7 @@
       <c r="A84" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="B84" s="10" t="s">
+      <c r="B84" s="17" t="s">
         <v>136</v>
       </c>
       <c r="C84" s="11" t="s">
@@ -6038,7 +6085,7 @@
       <c r="A85" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="B85" s="10" t="s">
+      <c r="B85" s="17" t="s">
         <v>136</v>
       </c>
       <c r="C85" s="11" t="s">
@@ -6099,7 +6146,7 @@
       <c r="A86" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="B86" s="10" t="s">
+      <c r="B86" s="17" t="s">
         <v>136</v>
       </c>
       <c r="C86" s="11" t="s">
@@ -6160,7 +6207,7 @@
       <c r="A87" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="B87" s="10" t="s">
+      <c r="B87" s="17" t="s">
         <v>140</v>
       </c>
       <c r="C87" s="11" t="s">
@@ -6221,7 +6268,7 @@
       <c r="A88" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="B88" s="10" t="s">
+      <c r="B88" s="17" t="s">
         <v>140</v>
       </c>
       <c r="C88" s="11" t="s">
@@ -6282,7 +6329,7 @@
       <c r="A89" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="B89" s="10" t="s">
+      <c r="B89" s="17" t="s">
         <v>137</v>
       </c>
       <c r="C89" s="11" t="s">
@@ -6343,7 +6390,7 @@
       <c r="A90" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="B90" s="10" t="s">
+      <c r="B90" s="17" t="s">
         <v>137</v>
       </c>
       <c r="C90" s="11" t="s">
@@ -6404,7 +6451,7 @@
       <c r="A91" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="B91" s="10" t="s">
+      <c r="B91" s="17" t="s">
         <v>137</v>
       </c>
       <c r="C91" s="11" t="s">
@@ -6465,7 +6512,7 @@
       <c r="A92" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="B92" s="10" t="s">
+      <c r="B92" s="17" t="s">
         <v>137</v>
       </c>
       <c r="C92" s="11" t="s">
@@ -6526,7 +6573,7 @@
       <c r="A93" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="B93" s="10" t="s">
+      <c r="B93" s="17" t="s">
         <v>137</v>
       </c>
       <c r="C93" s="11" t="s">
@@ -6587,7 +6634,7 @@
       <c r="A94" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="B94" s="10" t="s">
+      <c r="B94" s="17" t="s">
         <v>137</v>
       </c>
       <c r="C94" s="11" t="s">
@@ -6648,7 +6695,7 @@
       <c r="A95" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="B95" s="10" t="s">
+      <c r="B95" s="17" t="s">
         <v>137</v>
       </c>
       <c r="C95" s="11" t="s">
@@ -6709,7 +6756,7 @@
       <c r="A96" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="B96" s="10" t="s">
+      <c r="B96" s="17" t="s">
         <v>137</v>
       </c>
       <c r="C96" s="11" t="s">
@@ -6770,7 +6817,7 @@
       <c r="A97" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="B97" s="10" t="s">
+      <c r="B97" s="17" t="s">
         <v>137</v>
       </c>
       <c r="C97" s="11" t="s">
@@ -6831,7 +6878,7 @@
       <c r="A98" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="B98" s="10" t="s">
+      <c r="B98" s="17" t="s">
         <v>137</v>
       </c>
       <c r="C98" s="11" t="s">
@@ -6890,7 +6937,7 @@
     </row>
     <row r="99" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A99" s="10"/>
-      <c r="B99" s="10"/>
+      <c r="B99" s="17"/>
       <c r="C99" s="10"/>
       <c r="D99" s="6"/>
       <c r="E99" s="9"/>
@@ -6912,7 +6959,7 @@
     </row>
     <row r="100" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A100" s="10"/>
-      <c r="B100" s="10"/>
+      <c r="B100" s="17"/>
       <c r="C100" s="10"/>
       <c r="D100" s="6"/>
       <c r="E100" s="9"/>

</xml_diff>